<commit_message>
Phase 2 peers (MS, JPM, BEN) integrated; text-to-SQL agent, guardrail, gateway scaffolding
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/excel/AssetLens_PnL_Model.xlsx
+++ b/outputs/excel/AssetLens_PnL_Model.xlsx
@@ -3858,7 +3858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3937,46 +3937,43 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>BLK</t>
+          <t>BEN</t>
         </is>
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="C4" s="9" t="n">
-        <v>15488263</v>
+        <v>1791600</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>15.56737517800104</v>
+        <v>43.78678971810572</v>
       </c>
       <c r="E4" s="11" t="n">
-        <v>0.06451464594416437</v>
-      </c>
-      <c r="F4" s="11" t="n">
-        <v>0.3245743115408871</v>
+        <v>0.03834222608264053</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>0.3336486581178614</v>
+        <v>0.4246629701526153</v>
       </c>
       <c r="H4" s="22">
-        <f>IF(ISNUMBER(D4),(D4-AVERAGE(D$4:D$7))/STDEV(D$4:D$7),"")</f>
+        <f>IF(ISNUMBER(D4),(D4-AVERAGE(D$4:D$9))/STDEV(D$4:D$9),"")</f>
         <v/>
       </c>
       <c r="I4" s="22">
-        <f>IF(ISNUMBER(E4),(E4-AVERAGE(E$4:E$7))/STDEV(E$4:E$7),"")</f>
+        <f>IF(ISNUMBER(E4),(E4-AVERAGE(E$4:E$9))/STDEV(E$4:E$9),"")</f>
         <v/>
       </c>
       <c r="J4" s="22">
-        <f>IF(ISNUMBER(F4),(F4-AVERAGE(F$4:F$7))/STDEV(F$4:F$7),"")</f>
+        <f>IF(ISNUMBER(F4),(F4-AVERAGE(F$4:F$9))/STDEV(F$4:F$9),"")</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>BLK</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
@@ -3985,104 +3982,182 @@
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>4097000</v>
+        <v>15488263</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>34.7782237998872</v>
+        <v>15.56737517800104</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>0.1494785631517961</v>
+        <v>0.06451464594416437</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>0.3245743115408871</v>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>0.3336486581178614</v>
       </c>
       <c r="H5" s="22">
-        <f>IF(ISNUMBER(D5),(D5-AVERAGE(D$4:D$7))/STDEV(D$4:D$7),"")</f>
+        <f>IF(ISNUMBER(D5),(D5-AVERAGE(D$4:D$9))/STDEV(D$4:D$9),"")</f>
         <v/>
       </c>
       <c r="I5" s="22">
-        <f>IF(ISNUMBER(E5),(E5-AVERAGE(E$4:E$7))/STDEV(E$4:E$7),"")</f>
+        <f>IF(ISNUMBER(E5),(E5-AVERAGE(E$4:E$9))/STDEV(E$4:E$9),"")</f>
         <v/>
       </c>
       <c r="J5" s="22">
-        <f>IF(ISNUMBER(F5),(F5-AVERAGE(F$4:F$7))/STDEV(F$4:F$7),"")</f>
+        <f>IF(ISNUMBER(F5),(F5-AVERAGE(F$4:F$9))/STDEV(F$4:F$9),"")</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>IVZ</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C6" s="9" t="n">
-        <v>2470300</v>
+        <v>4097000</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>23.8735967491118</v>
+        <v>34.7782237998872</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>0.0762466273608474</v>
-      </c>
-      <c r="G6" s="11" t="n">
-        <v>0.3023831944947483</v>
+        <v>0.1494785631517961</v>
       </c>
       <c r="H6" s="22">
-        <f>IF(ISNUMBER(D6),(D6-AVERAGE(D$4:D$7))/STDEV(D$4:D$7),"")</f>
+        <f>IF(ISNUMBER(D6),(D6-AVERAGE(D$4:D$9))/STDEV(D$4:D$9),"")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>IF(ISNUMBER(E6),(E6-AVERAGE(E$4:E$7))/STDEV(E$4:E$7),"")</f>
+        <f>IF(ISNUMBER(E6),(E6-AVERAGE(E$4:E$9))/STDEV(E$4:E$9),"")</f>
         <v/>
       </c>
       <c r="J6" s="22">
-        <f>IF(ISNUMBER(F6),(F6-AVERAGE(F$4:F$7))/STDEV(F$4:F$7),"")</f>
+        <f>IF(ISNUMBER(F6),(F6-AVERAGE(F$4:F$9))/STDEV(F$4:F$9),"")</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>IVZ</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>2470300</v>
+      </c>
+      <c r="D7" s="36" t="n">
+        <v>23.8735967491118</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>0.0762466273608474</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>0.3023831944947483</v>
+      </c>
+      <c r="H7" s="22">
+        <f>IF(ISNUMBER(D7),(D7-AVERAGE(D$4:D$9))/STDEV(D$4:D$9),"")</f>
+        <v/>
+      </c>
+      <c r="I7" s="22">
+        <f>IF(ISNUMBER(E7),(E7-AVERAGE(E$4:E$9))/STDEV(E$4:E$9),"")</f>
+        <v/>
+      </c>
+      <c r="J7" s="22">
+        <f>IF(ISNUMBER(F7),(F7-AVERAGE(F$4:F$9))/STDEV(F$4:F$9),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>5140000</v>
+      </c>
+      <c r="D8" s="36" t="n">
+        <v>35.11323696519649</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>0.0932535113976514</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>0.3680009299802379</v>
+      </c>
+      <c r="G8" s="11" t="n">
+        <v>0.3525400085248189</v>
+      </c>
+      <c r="H8" s="22">
+        <f>IF(ISNUMBER(D8),(D8-AVERAGE(D$4:D$9))/STDEV(D$4:D$9),"")</f>
+        <v/>
+      </c>
+      <c r="I8" s="22">
+        <f>IF(ISNUMBER(E8),(E8-AVERAGE(E$4:E$9))/STDEV(E$4:E$9),"")</f>
+        <v/>
+      </c>
+      <c r="J8" s="22">
+        <f>IF(ISNUMBER(F8),(F8-AVERAGE(F$4:F$9))/STDEV(F$4:F$9),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>TROW</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C9" s="9" t="n">
         <v>1893400</v>
       </c>
-      <c r="D7" s="36" t="n">
+      <c r="D9" s="36" t="n">
         <v>38.60953693417518</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E9" s="11" t="n">
         <v>-0.03196564885496183</v>
       </c>
-      <c r="F7" s="11" t="n">
+      <c r="F9" s="11" t="n">
         <v>0.3075869336143309</v>
       </c>
-      <c r="G7" s="11" t="n">
+      <c r="G9" s="11" t="n">
         <v>0.3897523709167545</v>
       </c>
-      <c r="H7" s="22">
-        <f>IF(ISNUMBER(D7),(D7-AVERAGE(D$4:D$7))/STDEV(D$4:D$7),"")</f>
-        <v/>
-      </c>
-      <c r="I7" s="22">
-        <f>IF(ISNUMBER(E7),(E7-AVERAGE(E$4:E$7))/STDEV(E$4:E$7),"")</f>
-        <v/>
-      </c>
-      <c r="J7" s="22">
-        <f>IF(ISNUMBER(F7),(F7-AVERAGE(F$4:F$7))/STDEV(F$4:F$7),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="H9" s="22">
+        <f>IF(ISNUMBER(D9),(D9-AVERAGE(D$4:D$9))/STDEV(D$4:D$9),"")</f>
+        <v/>
+      </c>
+      <c r="I9" s="22">
+        <f>IF(ISNUMBER(E9),(E9-AVERAGE(E$4:E$9))/STDEV(E$4:E$9),"")</f>
+        <v/>
+      </c>
+      <c r="J9" s="22">
+        <f>IF(ISNUMBER(F9),(F9-AVERAGE(F$4:F$9))/STDEV(F$4:F$9),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Comparability: see warehouse table comparability_flags. GS = AWM segment/AUS; BLK = whole firm, residual market; IVZ gross fees; margins are GAAP-operating.</t>
         </is>
@@ -10887,29 +10962,29 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>LIQ</t>
+          <t>FIMA</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>343.9617177824462</v>
+        <v>2312.906455156511</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>214.7294957154298</v>
+        <v>1138.791729179275</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>89.56353791787843</v>
+        <v>601.9879101707099</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>69.58658111300879</v>
+        <v>632.2156216800502</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>283.971447855614</v>
+        <v>753.6458727246948</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>302.8058046386294</v>
+        <v>751.240604716781</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>299.0826981631084</v>
+        <v>751.9667663511592</v>
       </c>
       <c r="I6" s="18">
         <f>INDEX(D6:H6,MATCH($B$2,$D$4:$H$4,0))</f>
@@ -10935,29 +11010,29 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ALT</t>
+          <t>PBL</t>
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>4997.736800269337</v>
+        <v>3160</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>2687.535759907664</v>
+        <v>2046.357853093787</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>1296.734192728171</v>
+        <v>822.1958726036935</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>1243.954406348593</v>
+        <v>564.6534637187303</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>856.694543572237</v>
+        <v>751.4279663336786</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>846.7338268580123</v>
+        <v>803.201813070418</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>847.8829777261902</v>
+        <v>790.5880128725943</v>
       </c>
       <c r="I7" s="18">
         <f>INDEX(D7:H7,MATCH($B$2,$D$4:$H$4,0))</f>
@@ -10983,29 +11058,29 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>LIQ</t>
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>3085.495026791706</v>
+        <v>343.9617177824462</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>1438.097701764649</v>
+        <v>214.7294957154298</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>803.3178980678773</v>
+        <v>89.56353791787843</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>887.0600980914917</v>
+        <v>69.58658111300879</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>810.0290094153718</v>
+        <v>283.971447855614</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>800.8429762391819</v>
+        <v>302.8058046386294</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>801.660897569485</v>
+        <v>299.0826981631084</v>
       </c>
       <c r="I8" s="18">
         <f>INDEX(D8:H8,MATCH($B$2,$D$4:$H$4,0))</f>
@@ -11031,29 +11106,29 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>PBL</t>
+          <t>ALT</t>
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>3160</v>
+        <v>4997.736800269337</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>2046.357853093787</v>
+        <v>2687.535759907664</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>822.1958726036935</v>
+        <v>1296.734192728171</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>564.6534637187303</v>
+        <v>1243.954406348593</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>751.4279663336786</v>
+        <v>856.694543572237</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>803.201813070418</v>
+        <v>846.7338268580123</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>790.5880128725943</v>
+        <v>847.8829777261902</v>
       </c>
       <c r="I9" s="18">
         <f>INDEX(D9:H9,MATCH($B$2,$D$4:$H$4,0))</f>
@@ -11079,29 +11154,29 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>FIMA</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>2312.906455156511</v>
+        <v>3085.495026791706</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>1138.791729179275</v>
+        <v>1438.097701764649</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>601.9879101707099</v>
+        <v>803.3178980678773</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>632.2156216800502</v>
+        <v>887.0600980914917</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>753.6458727246948</v>
+        <v>810.0290094153718</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>751.240604716781</v>
+        <v>800.8429762391819</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>751.9667663511592</v>
+        <v>801.660897569485</v>
       </c>
       <c r="I10" s="18">
         <f>INDEX(D10:H10,MATCH($B$2,$D$4:$H$4,0))</f>

</xml_diff>

<commit_message>
MS (3 AUM layouts) and JPM (2019-26) parsers extended; comparability notes; rebuilt outputs
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/excel/AssetLens_PnL_Model.xlsx
+++ b/outputs/excel/AssetLens_PnL_Model.xlsx
@@ -3858,7 +3858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3958,15 +3958,15 @@
         <v>0.4246629701526153</v>
       </c>
       <c r="H4" s="22">
-        <f>IF(ISNUMBER(D4),(D4-AVERAGE(D$4:D$9))/STDEV(D$4:D$9),"")</f>
+        <f>IF(ISNUMBER(D4),(D4-AVERAGE(D$4:D$10))/STDEV(D$4:D$10),"")</f>
         <v/>
       </c>
       <c r="I4" s="22">
-        <f>IF(ISNUMBER(E4),(E4-AVERAGE(E$4:E$9))/STDEV(E$4:E$9),"")</f>
+        <f>IF(ISNUMBER(E4),(E4-AVERAGE(E$4:E$10))/STDEV(E$4:E$10),"")</f>
         <v/>
       </c>
       <c r="J4" s="22">
-        <f>IF(ISNUMBER(F4),(F4-AVERAGE(F$4:F$9))/STDEV(F$4:F$9),"")</f>
+        <f>IF(ISNUMBER(F4),(F4-AVERAGE(F$4:F$10))/STDEV(F$4:F$10),"")</f>
         <v/>
       </c>
     </row>
@@ -3997,15 +3997,15 @@
         <v>0.3336486581178614</v>
       </c>
       <c r="H5" s="22">
-        <f>IF(ISNUMBER(D5),(D5-AVERAGE(D$4:D$9))/STDEV(D$4:D$9),"")</f>
+        <f>IF(ISNUMBER(D5),(D5-AVERAGE(D$4:D$10))/STDEV(D$4:D$10),"")</f>
         <v/>
       </c>
       <c r="I5" s="22">
-        <f>IF(ISNUMBER(E5),(E5-AVERAGE(E$4:E$9))/STDEV(E$4:E$9),"")</f>
+        <f>IF(ISNUMBER(E5),(E5-AVERAGE(E$4:E$10))/STDEV(E$4:E$10),"")</f>
         <v/>
       </c>
       <c r="J5" s="22">
-        <f>IF(ISNUMBER(F5),(F5-AVERAGE(F$4:F$9))/STDEV(F$4:F$9),"")</f>
+        <f>IF(ISNUMBER(F5),(F5-AVERAGE(F$4:F$10))/STDEV(F$4:F$10),"")</f>
         <v/>
       </c>
     </row>
@@ -4030,15 +4030,15 @@
         <v>0.1494785631517961</v>
       </c>
       <c r="H6" s="22">
-        <f>IF(ISNUMBER(D6),(D6-AVERAGE(D$4:D$9))/STDEV(D$4:D$9),"")</f>
+        <f>IF(ISNUMBER(D6),(D6-AVERAGE(D$4:D$10))/STDEV(D$4:D$10),"")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>IF(ISNUMBER(E6),(E6-AVERAGE(E$4:E$9))/STDEV(E$4:E$9),"")</f>
+        <f>IF(ISNUMBER(E6),(E6-AVERAGE(E$4:E$10))/STDEV(E$4:E$10),"")</f>
         <v/>
       </c>
       <c r="J6" s="22">
-        <f>IF(ISNUMBER(F6),(F6-AVERAGE(F$4:F$9))/STDEV(F$4:F$9),"")</f>
+        <f>IF(ISNUMBER(F6),(F6-AVERAGE(F$4:F$10))/STDEV(F$4:F$10),"")</f>
         <v/>
       </c>
     </row>
@@ -4066,15 +4066,15 @@
         <v>0.3023831944947483</v>
       </c>
       <c r="H7" s="22">
-        <f>IF(ISNUMBER(D7),(D7-AVERAGE(D$4:D$9))/STDEV(D$4:D$9),"")</f>
+        <f>IF(ISNUMBER(D7),(D7-AVERAGE(D$4:D$10))/STDEV(D$4:D$10),"")</f>
         <v/>
       </c>
       <c r="I7" s="22">
-        <f>IF(ISNUMBER(E7),(E7-AVERAGE(E$4:E$9))/STDEV(E$4:E$9),"")</f>
+        <f>IF(ISNUMBER(E7),(E7-AVERAGE(E$4:E$10))/STDEV(E$4:E$10),"")</f>
         <v/>
       </c>
       <c r="J7" s="22">
-        <f>IF(ISNUMBER(F7),(F7-AVERAGE(F$4:F$9))/STDEV(F$4:F$9),"")</f>
+        <f>IF(ISNUMBER(F7),(F7-AVERAGE(F$4:F$10))/STDEV(F$4:F$10),"")</f>
         <v/>
       </c>
     </row>
@@ -4105,59 +4105,98 @@
         <v>0.3525400085248189</v>
       </c>
       <c r="H8" s="22">
-        <f>IF(ISNUMBER(D8),(D8-AVERAGE(D$4:D$9))/STDEV(D$4:D$9),"")</f>
+        <f>IF(ISNUMBER(D8),(D8-AVERAGE(D$4:D$10))/STDEV(D$4:D$10),"")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>IF(ISNUMBER(E8),(E8-AVERAGE(E$4:E$9))/STDEV(E$4:E$9),"")</f>
+        <f>IF(ISNUMBER(E8),(E8-AVERAGE(E$4:E$10))/STDEV(E$4:E$10),"")</f>
         <v/>
       </c>
       <c r="J8" s="22">
-        <f>IF(ISNUMBER(F8),(F8-AVERAGE(F$4:F$9))/STDEV(F$4:F$9),"")</f>
+        <f>IF(ISNUMBER(F8),(F8-AVERAGE(F$4:F$10))/STDEV(F$4:F$10),"")</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>2004000</v>
+      </c>
+      <c r="D9" s="36" t="n">
+        <v>33.35801305781786</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>0.1009924109748978</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>0.2313797313797314</v>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>0.3646214896214896</v>
+      </c>
+      <c r="H9" s="22">
+        <f>IF(ISNUMBER(D9),(D9-AVERAGE(D$4:D$10))/STDEV(D$4:D$10),"")</f>
+        <v/>
+      </c>
+      <c r="I9" s="22">
+        <f>IF(ISNUMBER(E9),(E9-AVERAGE(E$4:E$10))/STDEV(E$4:E$10),"")</f>
+        <v/>
+      </c>
+      <c r="J9" s="22">
+        <f>IF(ISNUMBER(F9),(F9-AVERAGE(F$4:F$10))/STDEV(F$4:F$10),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>TROW</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C10" s="9" t="n">
         <v>1893400</v>
       </c>
-      <c r="D9" s="36" t="n">
+      <c r="D10" s="36" t="n">
         <v>38.60953693417518</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E10" s="11" t="n">
         <v>-0.03196564885496183</v>
       </c>
-      <c r="F9" s="11" t="n">
+      <c r="F10" s="11" t="n">
         <v>0.3075869336143309</v>
       </c>
-      <c r="G9" s="11" t="n">
+      <c r="G10" s="11" t="n">
         <v>0.3897523709167545</v>
       </c>
-      <c r="H9" s="22">
-        <f>IF(ISNUMBER(D9),(D9-AVERAGE(D$4:D$9))/STDEV(D$4:D$9),"")</f>
-        <v/>
-      </c>
-      <c r="I9" s="22">
-        <f>IF(ISNUMBER(E9),(E9-AVERAGE(E$4:E$9))/STDEV(E$4:E$9),"")</f>
-        <v/>
-      </c>
-      <c r="J9" s="22">
-        <f>IF(ISNUMBER(F9),(F9-AVERAGE(F$4:F$9))/STDEV(F$4:F$9),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="H10" s="22">
+        <f>IF(ISNUMBER(D10),(D10-AVERAGE(D$4:D$10))/STDEV(D$4:D$10),"")</f>
+        <v/>
+      </c>
+      <c r="I10" s="22">
+        <f>IF(ISNUMBER(E10),(E10-AVERAGE(E$4:E$10))/STDEV(E$4:E$10),"")</f>
+        <v/>
+      </c>
+      <c r="J10" s="22">
+        <f>IF(ISNUMBER(F10),(F10-AVERAGE(F$4:F$10))/STDEV(F$4:F$10),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Comparability: see warehouse table comparability_flags. GS = AWM segment/AUS; BLK = whole firm, residual market; IVZ gross fees; margins are GAAP-operating.</t>
         </is>
@@ -10914,29 +10953,29 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>PWM</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>3996.9</v>
+        <v>3085.495026791706</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>1664.087460339194</v>
+        <v>1438.097701764649</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>1039.80058851167</v>
+        <v>803.3178980678773</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1256.129829048126</v>
+        <v>887.0600980914917</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>1197.831160098404</v>
+        <v>810.0290094153718</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>1148.774974476977</v>
+        <v>800.8429762391819</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>1162.418647317463</v>
+        <v>801.660897569485</v>
       </c>
       <c r="I5" s="18">
         <f>INDEX(D5:H5,MATCH($B$2,$D$4:$H$4,0))</f>
@@ -10962,29 +11001,29 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>FIMA</t>
+          <t>PWM</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>2312.906455156511</v>
+        <v>3996.9</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>1138.791729179275</v>
+        <v>1664.087460339194</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>601.9879101707099</v>
+        <v>1039.80058851167</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>632.2156216800502</v>
+        <v>1256.129829048126</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>753.6458727246948</v>
+        <v>1197.831160098404</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>751.240604716781</v>
+        <v>1148.774974476977</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>751.9667663511592</v>
+        <v>1162.418647317463</v>
       </c>
       <c r="I6" s="18">
         <f>INDEX(D6:H6,MATCH($B$2,$D$4:$H$4,0))</f>
@@ -11058,29 +11097,29 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>LIQ</t>
+          <t>FIMA</t>
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>343.9617177824462</v>
+        <v>2312.906455156511</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>214.7294957154298</v>
+        <v>1138.791729179275</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>89.56353791787843</v>
+        <v>601.9879101707099</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>69.58658111300879</v>
+        <v>632.2156216800502</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>283.971447855614</v>
+        <v>753.6458727246948</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>302.8058046386294</v>
+        <v>751.240604716781</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>299.0826981631084</v>
+        <v>751.9667663511592</v>
       </c>
       <c r="I8" s="18">
         <f>INDEX(D8:H8,MATCH($B$2,$D$4:$H$4,0))</f>
@@ -11106,29 +11145,29 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ALT</t>
+          <t>LIQ</t>
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>4997.736800269337</v>
+        <v>343.9617177824462</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>2687.535759907664</v>
+        <v>214.7294957154298</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>1296.734192728171</v>
+        <v>89.56353791787843</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>1243.954406348593</v>
+        <v>69.58658111300879</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>856.694543572237</v>
+        <v>283.971447855614</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>846.7338268580123</v>
+        <v>302.8058046386294</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>847.8829777261902</v>
+        <v>299.0826981631084</v>
       </c>
       <c r="I9" s="18">
         <f>INDEX(D9:H9,MATCH($B$2,$D$4:$H$4,0))</f>
@@ -11154,29 +11193,29 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>ALT</t>
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>3085.495026791706</v>
+        <v>4997.736800269337</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>1438.097701764649</v>
+        <v>2687.535759907664</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>803.3178980678773</v>
+        <v>1296.734192728171</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>887.0600980914917</v>
+        <v>1243.954406348593</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>810.0290094153718</v>
+        <v>856.694543572237</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>800.8429762391819</v>
+        <v>846.7338268580123</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>801.660897569485</v>
+        <v>847.8829777261902</v>
       </c>
       <c r="I10" s="18">
         <f>INDEX(D10:H10,MATCH($B$2,$D$4:$H$4,0))</f>

</xml_diff>

<commit_message>
Close TROW/BEN/JPM parser gaps (acquired-AUM rows, long-term detail rows, JPM 10-K Q4 derivation); rebuilt outputs
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/excel/AssetLens_PnL_Model.xlsx
+++ b/outputs/excel/AssetLens_PnL_Model.xlsx
@@ -10953,29 +10953,29 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>LIQ</t>
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>3085.495026791706</v>
+        <v>343.9617177824462</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>1438.097701764649</v>
+        <v>214.7294957154298</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>803.3178980678773</v>
+        <v>89.56353791787843</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>887.0600980914917</v>
+        <v>69.58658111300879</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>810.0290094153718</v>
+        <v>283.971447855614</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>800.8429762391819</v>
+        <v>302.8058046386294</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>801.660897569485</v>
+        <v>299.0826981631084</v>
       </c>
       <c r="I5" s="18">
         <f>INDEX(D5:H5,MATCH($B$2,$D$4:$H$4,0))</f>
@@ -11001,29 +11001,29 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>PWM</t>
+          <t>ALT</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>3996.9</v>
+        <v>4997.736800269337</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>1664.087460339194</v>
+        <v>2687.535759907664</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>1039.80058851167</v>
+        <v>1296.734192728171</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>1256.129829048126</v>
+        <v>1243.954406348593</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>1197.831160098404</v>
+        <v>856.694543572237</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>1148.774974476977</v>
+        <v>846.7338268580123</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>1162.418647317463</v>
+        <v>847.8829777261902</v>
       </c>
       <c r="I6" s="18">
         <f>INDEX(D6:H6,MATCH($B$2,$D$4:$H$4,0))</f>
@@ -11097,29 +11097,29 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>FIMA</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>2312.906455156511</v>
+        <v>3085.495026791706</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>1138.791729179275</v>
+        <v>1438.097701764649</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>601.9879101707099</v>
+        <v>803.3178980678773</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>632.2156216800502</v>
+        <v>887.0600980914917</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>753.6458727246948</v>
+        <v>810.0290094153718</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>751.240604716781</v>
+        <v>800.8429762391819</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>751.9667663511592</v>
+        <v>801.660897569485</v>
       </c>
       <c r="I8" s="18">
         <f>INDEX(D8:H8,MATCH($B$2,$D$4:$H$4,0))</f>
@@ -11145,29 +11145,29 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>LIQ</t>
+          <t>FIMA</t>
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>343.9617177824462</v>
+        <v>2312.906455156511</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>214.7294957154298</v>
+        <v>1138.791729179275</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>89.56353791787843</v>
+        <v>601.9879101707099</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>69.58658111300879</v>
+        <v>632.2156216800502</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>283.971447855614</v>
+        <v>753.6458727246948</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>302.8058046386294</v>
+        <v>751.240604716781</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>299.0826981631084</v>
+        <v>751.9667663511592</v>
       </c>
       <c r="I9" s="18">
         <f>INDEX(D9:H9,MATCH($B$2,$D$4:$H$4,0))</f>
@@ -11193,29 +11193,29 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ALT</t>
+          <t>PWM</t>
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>4997.736800269337</v>
+        <v>3996.9</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>2687.535759907664</v>
+        <v>1664.087460339194</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>1296.734192728171</v>
+        <v>1039.80058851167</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>1243.954406348593</v>
+        <v>1256.129829048126</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>856.694543572237</v>
+        <v>1197.831160098404</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>846.7338268580123</v>
+        <v>1148.774974476977</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>847.8829777261902</v>
+        <v>1162.418647317463</v>
       </c>
       <c r="I10" s="18">
         <f>INDEX(D10:H10,MATCH($B$2,$D$4:$H$4,0))</f>

</xml_diff>

<commit_message>
Complete Morgan Stanley Investment Management P&L (2019-26) incl. derived Q4s; refresh outputs and README
</commit_message>
<xml_diff>
--- a/outputs/excel/AssetLens_PnL_Model.xlsx
+++ b/outputs/excel/AssetLens_PnL_Model.xlsx
@@ -552,7 +552,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>1.0 (Phase 1) - built 2026-10-21</t>
+          <t>1.0 (Phase 1) - built 2026-10-22</t>
         </is>
       </c>
     </row>
@@ -10953,29 +10953,29 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>LIQ</t>
+          <t>FIMA</t>
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>343.9617177824462</v>
+        <v>2312.906455156511</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>214.7294957154298</v>
+        <v>1138.791729179275</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>89.56353791787843</v>
+        <v>601.9879101707099</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>69.58658111300879</v>
+        <v>632.2156216800502</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>283.971447855614</v>
+        <v>753.6458727246948</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>302.8058046386294</v>
+        <v>751.240604716781</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>299.0826981631084</v>
+        <v>751.9667663511592</v>
       </c>
       <c r="I5" s="18">
         <f>INDEX(D5:H5,MATCH($B$2,$D$4:$H$4,0))</f>
@@ -11001,29 +11001,29 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ALT</t>
+          <t>PWM</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>4997.736800269337</v>
+        <v>3996.9</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>2687.535759907664</v>
+        <v>1664.087460339194</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>1296.734192728171</v>
+        <v>1039.80058851167</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>1243.954406348593</v>
+        <v>1256.129829048126</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>856.694543572237</v>
+        <v>1197.831160098404</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>846.7338268580123</v>
+        <v>1148.774974476977</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>847.8829777261902</v>
+        <v>1162.418647317463</v>
       </c>
       <c r="I6" s="18">
         <f>INDEX(D6:H6,MATCH($B$2,$D$4:$H$4,0))</f>
@@ -11049,29 +11049,29 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>FIMA</t>
+          <t>LIQ</t>
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>2312.906455156511</v>
+        <v>343.9617177824462</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>1138.791729179275</v>
+        <v>214.7294957154298</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>601.9879101707099</v>
+        <v>89.56353791787843</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>632.2156216800502</v>
+        <v>69.58658111300879</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>753.6458727246948</v>
+        <v>283.971447855614</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>751.240604716781</v>
+        <v>302.8058046386294</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>751.9667663511592</v>
+        <v>299.0826981631084</v>
       </c>
       <c r="I7" s="18">
         <f>INDEX(D7:H7,MATCH($B$2,$D$4:$H$4,0))</f>
@@ -11097,29 +11097,29 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>PWM</t>
+          <t>ALT</t>
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>3996.9</v>
+        <v>4997.736800269337</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>1664.087460339194</v>
+        <v>2687.535759907664</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>1039.80058851167</v>
+        <v>1296.734192728171</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>1256.129829048126</v>
+        <v>1243.954406348593</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>1197.831160098404</v>
+        <v>856.694543572237</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>1148.774974476977</v>
+        <v>846.7338268580123</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>1162.418647317463</v>
+        <v>847.8829777261902</v>
       </c>
       <c r="I8" s="18">
         <f>INDEX(D8:H8,MATCH($B$2,$D$4:$H$4,0))</f>

</xml_diff>